<commit_message>
WOrk on cattle feed rations
</commit_message>
<xml_diff>
--- a/data/prod_parameters/PigHerd.xlsx
+++ b/data/prod_parameters/PigHerd.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="9000"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="9000" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="default" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="735" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="727" uniqueCount="246">
   <si>
     <t>parameter</t>
   </si>
@@ -728,36 +728,6 @@
     <t>barley brewers grain</t>
   </si>
   <si>
-    <t>Sojamjöl, 45% Rp i vara</t>
-  </si>
-  <si>
-    <t>Sojaprotein-Hamlet 310</t>
-  </si>
-  <si>
-    <t>http://www2.freefarm.se/fodertabell/fodtab.pl?djur=gris</t>
-  </si>
-  <si>
-    <t>Palmkärnkaka</t>
-  </si>
-  <si>
-    <t>Agrodrank10</t>
-  </si>
-  <si>
-    <t>Agrodrank90</t>
-  </si>
-  <si>
-    <t>Betfiber, omelasserad</t>
-  </si>
-  <si>
-    <t>Vasslepulver, söt vassle</t>
-  </si>
-  <si>
-    <t>Potatisproteinkoncentrat</t>
-  </si>
-  <si>
-    <t>Potato protein concentrate is a byproduct of potato starch production</t>
-  </si>
-  <si>
     <t>sows, gilts</t>
   </si>
   <si>
@@ -798,6 +768,54 @@
   </si>
   <si>
     <t>excluded</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Etanolindustri: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Ts-halten varierar mellan 8–27% på de produkter vi har räknat med, fyra olika drank: St1, Agroetanol, Drank Skåne och Drank Lidköping. Baserat på svaren från foderoptimerarna räknade vi ut en medel-ts på 8,7% och volymen 306 447 ton. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Mejerindustri:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Ts-halten varierar mellan 5–16 % på de produkter vi har räknat med. Det är fodermjölk, permeat och vassle från cirka 10 mejerier. Medel-ts blev 7,8 % och mängden 317 407 ton. </t>
+    </r>
+  </si>
+  <si>
+    <t>E-mail from Birgit Landquist (RISE) 2023-10-16</t>
   </si>
 </sst>
 </file>
@@ -810,7 +828,7 @@
     <numFmt numFmtId="166" formatCode="#,##0.000"/>
     <numFmt numFmtId="167" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -950,6 +968,21 @@
       <b/>
       <i/>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1284,7 +1317,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="154">
+  <cellXfs count="165">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1529,7 +1562,6 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="21" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1539,9 +1571,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="20" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -1609,6 +1638,29 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="15" fillId="0" borderId="22" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="15" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="15" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
@@ -8050,7 +8102,7 @@
       <c r="E54" s="8"/>
       <c r="F54" s="8"/>
       <c r="G54" s="8" t="s">
-        <v>245</v>
+        <v>235</v>
       </c>
       <c r="H54" s="8" t="s">
         <v>159</v>
@@ -8121,7 +8173,7 @@
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" s="93" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="B60" s="93"/>
       <c r="C60" s="93"/>
@@ -8139,7 +8191,7 @@
         <v>71</v>
       </c>
       <c r="E61" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C61,'feed rations'!$K$8:$K$43,0),MATCH(B61,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C61,'feed rations'!$L$8:$L$43,0),MATCH(B61,'feed rations'!$Q$7:$T$7,0))</f>
         <v>39.939446969082496</v>
       </c>
       <c r="F61" t="s">
@@ -8154,7 +8206,7 @@
         <v>71</v>
       </c>
       <c r="E62" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C62,'feed rations'!$K$8:$K$43,0),MATCH(B62,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C62,'feed rations'!$L$8:$L$43,0),MATCH(B62,'feed rations'!$Q$7:$T$7,0))</f>
         <v>33.588951440574981</v>
       </c>
       <c r="F62" t="s">
@@ -8169,7 +8221,7 @@
         <v>71</v>
       </c>
       <c r="E63" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C63,'feed rations'!$K$8:$K$43,0),MATCH(B63,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C63,'feed rations'!$L$8:$L$43,0),MATCH(B63,'feed rations'!$Q$7:$T$7,0))</f>
         <v>4.876686724200181</v>
       </c>
       <c r="F63" t="s">
@@ -8184,7 +8236,7 @@
         <v>71</v>
       </c>
       <c r="E64" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C64,'feed rations'!$K$8:$K$43,0),MATCH(B64,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C64,'feed rations'!$L$8:$L$43,0),MATCH(B64,'feed rations'!$Q$7:$T$7,0))</f>
         <v>0.44754403481583932</v>
       </c>
       <c r="F64" t="s">
@@ -8199,7 +8251,7 @@
         <v>71</v>
       </c>
       <c r="E65" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C65,'feed rations'!$K$8:$K$43,0),MATCH(B65,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C65,'feed rations'!$L$8:$L$43,0),MATCH(B65,'feed rations'!$Q$7:$T$7,0))</f>
         <v>0.22377201740791966</v>
       </c>
       <c r="F65" t="s">
@@ -8214,7 +8266,7 @@
         <v>71</v>
       </c>
       <c r="E66" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C66,'feed rations'!$K$8:$K$43,0),MATCH(B66,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C66,'feed rations'!$L$8:$L$43,0),MATCH(B66,'feed rations'!$Q$7:$T$7,0))</f>
         <v>0.78553488869540378</v>
       </c>
       <c r="F66" t="s">
@@ -8229,7 +8281,7 @@
         <v>71</v>
       </c>
       <c r="E67" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C67,'feed rations'!$K$8:$K$43,0),MATCH(B67,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C67,'feed rations'!$L$8:$L$43,0),MATCH(B67,'feed rations'!$Q$7:$T$7,0))</f>
         <v>9.9145180126604351E-2</v>
       </c>
       <c r="F67" t="s">
@@ -8244,7 +8296,7 @@
         <v>71</v>
       </c>
       <c r="E68" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C68,'feed rations'!$K$8:$K$43,0),MATCH(B68,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C68,'feed rations'!$L$8:$L$43,0),MATCH(B68,'feed rations'!$Q$7:$T$7,0))</f>
         <v>0.35109057903656365</v>
       </c>
       <c r="F68" t="s">
@@ -8259,7 +8311,7 @@
         <v>71</v>
       </c>
       <c r="E69" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C69,'feed rations'!$K$8:$K$43,0),MATCH(B69,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C69,'feed rations'!$L$8:$L$43,0),MATCH(B69,'feed rations'!$Q$7:$T$7,0))</f>
         <v>0.13063835499034929</v>
       </c>
       <c r="F69" t="s">
@@ -8268,13 +8320,13 @@
     </row>
     <row r="70" spans="3:6" x14ac:dyDescent="0.25">
       <c r="C70" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
       <c r="D70" t="s">
         <v>71</v>
       </c>
       <c r="E70" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C70,'feed rations'!$K$8:$K$43,0),MATCH(B70,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C70,'feed rations'!$L$8:$L$43,0),MATCH(B70,'feed rations'!$Q$7:$T$7,0))</f>
         <v>0.20636553329519458</v>
       </c>
       <c r="F70" t="s">
@@ -8289,7 +8341,7 @@
         <v>71</v>
       </c>
       <c r="E71" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C71,'feed rations'!$K$8:$K$43,0),MATCH(B71,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C71,'feed rations'!$L$8:$L$43,0),MATCH(B71,'feed rations'!$Q$7:$T$7,0))</f>
         <v>6.9956121304172738</v>
       </c>
       <c r="F71" t="s">
@@ -8304,7 +8356,7 @@
         <v>71</v>
       </c>
       <c r="E72" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C72,'feed rations'!$K$8:$K$43,0),MATCH(B72,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C72,'feed rations'!$L$8:$L$43,0),MATCH(B72,'feed rations'!$Q$7:$T$7,0))</f>
         <v>3.2865954280882512</v>
       </c>
       <c r="F72" t="s">
@@ -8319,7 +8371,7 @@
         <v>71</v>
       </c>
       <c r="E73" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C73,'feed rations'!$K$8:$K$43,0),MATCH(B73,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C73,'feed rations'!$L$8:$L$43,0),MATCH(B73,'feed rations'!$Q$7:$T$7,0))</f>
         <v>0.44906934527932563</v>
       </c>
       <c r="F73" t="s">
@@ -8334,7 +8386,7 @@
         <v>71</v>
       </c>
       <c r="E74" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C74,'feed rations'!$K$8:$K$43,0),MATCH(B74,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C74,'feed rations'!$L$8:$L$43,0),MATCH(B74,'feed rations'!$Q$7:$T$7,0))</f>
         <v>0.13063835499034929</v>
       </c>
       <c r="F74" t="s">
@@ -8349,7 +8401,7 @@
         <v>71</v>
       </c>
       <c r="E75" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C75,'feed rations'!$K$8:$K$43,0),MATCH(B75,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C75,'feed rations'!$L$8:$L$43,0),MATCH(B75,'feed rations'!$Q$7:$T$7,0))</f>
         <v>3.1145942422939523</v>
       </c>
       <c r="F75" t="s">
@@ -8364,7 +8416,7 @@
         <v>71</v>
       </c>
       <c r="E76" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C76,'feed rations'!$K$8:$K$43,0),MATCH(B76,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C76,'feed rations'!$L$8:$L$43,0),MATCH(B76,'feed rations'!$Q$7:$T$7,0))</f>
         <v>2.3450302513926982</v>
       </c>
       <c r="F76" t="s">
@@ -8379,7 +8431,7 @@
         <v>71</v>
       </c>
       <c r="E77" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C77,'feed rations'!$K$8:$K$43,0),MATCH(B77,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C77,'feed rations'!$L$8:$L$43,0),MATCH(B77,'feed rations'!$Q$7:$T$7,0))</f>
         <v>0.13727794171375987</v>
       </c>
       <c r="F77" t="s">
@@ -8394,7 +8446,7 @@
         <v>71</v>
       </c>
       <c r="E78" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C78,'feed rations'!$K$8:$K$43,0),MATCH(B78,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C78,'feed rations'!$L$8:$L$43,0),MATCH(B78,'feed rations'!$Q$7:$T$7,0))</f>
         <v>0.59612721878837949</v>
       </c>
       <c r="F78" t="s">
@@ -8409,7 +8461,7 @@
         <v>71</v>
       </c>
       <c r="E79" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C79,'feed rations'!$K$8:$K$43,0),MATCH(B79,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C79,'feed rations'!$L$8:$L$43,0),MATCH(B79,'feed rations'!$Q$7:$T$7,0))</f>
         <v>0.35458982068809092</v>
       </c>
       <c r="F79" t="s">
@@ -8424,7 +8476,7 @@
         <v>71</v>
       </c>
       <c r="E80" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C80,'feed rations'!$K$8:$K$43,0),MATCH(B80,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C80,'feed rations'!$L$8:$L$43,0),MATCH(B80,'feed rations'!$Q$7:$T$7,0))</f>
         <v>0.69473405404551813</v>
       </c>
       <c r="F80" t="s">
@@ -8439,7 +8491,7 @@
         <v>71</v>
       </c>
       <c r="E81" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C81,'feed rations'!$K$8:$K$43,0),MATCH(B81,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C81,'feed rations'!$L$8:$L$43,0),MATCH(B81,'feed rations'!$Q$7:$T$7,0))</f>
         <v>1.0649538207770974</v>
       </c>
       <c r="F81" t="s">
@@ -8454,7 +8506,7 @@
         <v>71</v>
       </c>
       <c r="E82" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C82,'feed rations'!$K$8:$K$43,0),MATCH(B82,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C82,'feed rations'!$L$8:$L$43,0),MATCH(B82,'feed rations'!$Q$7:$T$7,0))</f>
         <v>0.18160166929977128</v>
       </c>
       <c r="F82" t="s">
@@ -8463,7 +8515,7 @@
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83" s="93" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="B83" s="93"/>
       <c r="C83" s="93"/>
@@ -8484,7 +8536,7 @@
         <v>71</v>
       </c>
       <c r="E84" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C84,'feed rations'!$K$8:$K$43,0),MATCH(B84,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C84,'feed rations'!$L$8:$L$43,0),MATCH(B84,'feed rations'!$Q$7:$T$7,0))</f>
         <v>37.344664381805039</v>
       </c>
       <c r="F84" t="s">
@@ -8502,7 +8554,7 @@
         <v>71</v>
       </c>
       <c r="E85" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C85,'feed rations'!$K$8:$K$43,0),MATCH(B85,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C85,'feed rations'!$L$8:$L$43,0),MATCH(B85,'feed rations'!$Q$7:$T$7,0))</f>
         <v>33.835769741903896</v>
       </c>
       <c r="F85" t="s">
@@ -8520,7 +8572,7 @@
         <v>71</v>
       </c>
       <c r="E86" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C86,'feed rations'!$K$8:$K$43,0),MATCH(B86,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C86,'feed rations'!$L$8:$L$43,0),MATCH(B86,'feed rations'!$Q$7:$T$7,0))</f>
         <v>7.2684246112238</v>
       </c>
       <c r="F86" t="s">
@@ -8538,7 +8590,7 @@
         <v>71</v>
       </c>
       <c r="E87" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C87,'feed rations'!$K$8:$K$43,0),MATCH(B87,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C87,'feed rations'!$L$8:$L$43,0),MATCH(B87,'feed rations'!$Q$7:$T$7,0))</f>
         <v>1.7544473199505721</v>
       </c>
       <c r="F87" t="s">
@@ -8556,7 +8608,7 @@
         <v>71</v>
       </c>
       <c r="E88" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C88,'feed rations'!$K$8:$K$43,0),MATCH(B88,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C88,'feed rations'!$L$8:$L$43,0),MATCH(B88,'feed rations'!$Q$7:$T$7,0))</f>
         <v>0.24772096710265556</v>
       </c>
       <c r="F88" t="s">
@@ -8574,7 +8626,7 @@
         <v>71</v>
       </c>
       <c r="E89" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C89,'feed rations'!$K$8:$K$43,0),MATCH(B89,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C89,'feed rations'!$L$8:$L$43,0),MATCH(B89,'feed rations'!$Q$7:$T$7,0))</f>
         <v>0.74316290130796658</v>
       </c>
       <c r="F89" t="s">
@@ -8586,13 +8638,13 @@
         <v>15</v>
       </c>
       <c r="C90" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
       <c r="D90" t="s">
         <v>71</v>
       </c>
       <c r="E90" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C90,'feed rations'!$K$8:$K$43,0),MATCH(B90,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C90,'feed rations'!$L$8:$L$43,0),MATCH(B90,'feed rations'!$Q$7:$T$7,0))</f>
         <v>1.4571821594273857</v>
       </c>
       <c r="F90" t="s">
@@ -8610,7 +8662,7 @@
         <v>71</v>
       </c>
       <c r="E91" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C91,'feed rations'!$K$8:$K$43,0),MATCH(B91,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C91,'feed rations'!$L$8:$L$43,0),MATCH(B91,'feed rations'!$Q$7:$T$7,0))</f>
         <v>7.1809936816581557</v>
       </c>
       <c r="F91" t="s">
@@ -8628,7 +8680,7 @@
         <v>71</v>
       </c>
       <c r="E92" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C92,'feed rations'!$K$8:$K$43,0),MATCH(B92,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C92,'feed rations'!$L$8:$L$43,0),MATCH(B92,'feed rations'!$Q$7:$T$7,0))</f>
         <v>2.2819472616632859</v>
       </c>
       <c r="F92" t="s">
@@ -8646,7 +8698,7 @@
         <v>71</v>
       </c>
       <c r="E93" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C93,'feed rations'!$K$8:$K$43,0),MATCH(B93,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C93,'feed rations'!$L$8:$L$43,0),MATCH(B93,'feed rations'!$Q$7:$T$7,0))</f>
         <v>1.2823203002960992</v>
       </c>
       <c r="F93" t="s">
@@ -8664,7 +8716,7 @@
         <v>71</v>
       </c>
       <c r="E94" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C94,'feed rations'!$K$8:$K$43,0),MATCH(B94,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C94,'feed rations'!$L$8:$L$43,0),MATCH(B94,'feed rations'!$Q$7:$T$7,0))</f>
         <v>1.7626075400433656</v>
       </c>
       <c r="F94" t="s">
@@ -8676,13 +8728,13 @@
         <v>15</v>
       </c>
       <c r="C95" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="D95" t="s">
         <v>71</v>
       </c>
       <c r="E95" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C95,'feed rations'!$K$8:$K$43,0),MATCH(B95,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C95,'feed rations'!$L$8:$L$43,0),MATCH(B95,'feed rations'!$Q$7:$T$7,0))</f>
         <v>0.2826933389289128</v>
       </c>
       <c r="F95" t="s">
@@ -8700,7 +8752,7 @@
         <v>71</v>
       </c>
       <c r="E96" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C96,'feed rations'!$K$8:$K$43,0),MATCH(B96,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C96,'feed rations'!$L$8:$L$43,0),MATCH(B96,'feed rations'!$Q$7:$T$7,0))</f>
         <v>1.3406075866731948</v>
       </c>
       <c r="F96" t="s">
@@ -8718,7 +8770,7 @@
         <v>71</v>
       </c>
       <c r="E97" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C97,'feed rations'!$K$8:$K$43,0),MATCH(B97,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C97,'feed rations'!$L$8:$L$43,0),MATCH(B97,'feed rations'!$Q$7:$T$7,0))</f>
         <v>3.2174582080156675</v>
       </c>
       <c r="F97" t="s">
@@ -8727,7 +8779,7 @@
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A98" s="93" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="B98" s="93"/>
       <c r="C98" s="93"/>
@@ -8748,8 +8800,8 @@
         <v>71</v>
       </c>
       <c r="E99" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C99,'feed rations'!$K$8:$K$43,0),MATCH(B99,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>21.826284108458598</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C99,'feed rations'!$L$8:$L$43,0),MATCH(B99,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>31.302145183860713</v>
       </c>
       <c r="F99" t="s">
         <v>23</v>
@@ -8766,8 +8818,8 @@
         <v>71</v>
       </c>
       <c r="E100" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C100,'feed rations'!$K$8:$K$43,0),MATCH(B100,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>16.76667694151628</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C100,'feed rations'!$L$8:$L$43,0),MATCH(B100,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>24.045914241116183</v>
       </c>
       <c r="F100" t="s">
         <v>23</v>
@@ -8784,8 +8836,8 @@
         <v>71</v>
       </c>
       <c r="E101" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C101,'feed rations'!$K$8:$K$43,0),MATCH(B101,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>2.8258444283454405</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C101,'feed rations'!$L$8:$L$43,0),MATCH(B101,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>4.0526821754690197</v>
       </c>
       <c r="F101" t="s">
         <v>23</v>
@@ -8802,8 +8854,8 @@
         <v>71</v>
       </c>
       <c r="E102" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C102,'feed rations'!$K$8:$K$43,0),MATCH(B102,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>2.6374547997890785</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C102,'feed rations'!$L$8:$L$43,0),MATCH(B102,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>3.7825033637710859</v>
       </c>
       <c r="F102" t="s">
         <v>23</v>
@@ -8820,8 +8872,8 @@
         <v>71</v>
       </c>
       <c r="E103" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C103,'feed rations'!$K$8:$K$43,0),MATCH(B103,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>5.3825608158960786E-2</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C103,'feed rations'!$L$8:$L$43,0),MATCH(B103,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>7.7193946199409905E-2</v>
       </c>
       <c r="F103" t="s">
         <v>23</v>
@@ -8838,8 +8890,8 @@
         <v>71</v>
       </c>
       <c r="E104" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C104,'feed rations'!$K$8:$K$43,0),MATCH(B104,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>0.31919837396593026</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C104,'feed rations'!$L$8:$L$43,0),MATCH(B104,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>0.45777805304301217</v>
       </c>
       <c r="F104" t="s">
         <v>23</v>
@@ -8856,8 +8908,8 @@
         <v>71</v>
       </c>
       <c r="E105" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C105,'feed rations'!$K$8:$K$43,0),MATCH(B105,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>5.3997724929236526</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C105,'feed rations'!$L$8:$L$43,0),MATCH(B105,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>7.74407873064429</v>
       </c>
       <c r="F105" t="s">
         <v>23</v>
@@ -8874,8 +8926,8 @@
         <v>71</v>
       </c>
       <c r="E106" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C106,'feed rations'!$K$8:$K$43,0),MATCH(B106,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>1.9827851935766017</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C106,'feed rations'!$L$8:$L$43,0),MATCH(B106,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>2.8436095530201233</v>
       </c>
       <c r="F106" t="s">
         <v>23</v>
@@ -8892,8 +8944,8 @@
         <v>71</v>
       </c>
       <c r="E107" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C107,'feed rations'!$K$8:$K$43,0),MATCH(B107,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>2.4503169295619931</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C107,'feed rations'!$L$8:$L$43,0),MATCH(B107,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>3.5141197601242991</v>
       </c>
       <c r="F107" t="s">
         <v>23</v>
@@ -8910,8 +8962,8 @@
         <v>71</v>
       </c>
       <c r="E108" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C108,'feed rations'!$K$8:$K$43,0),MATCH(B108,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>0.11391000796431236</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C108,'feed rations'!$L$8:$L$43,0),MATCH(B108,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>0.16336393265456514</v>
       </c>
       <c r="F108" t="s">
         <v>23</v>
@@ -8928,8 +8980,8 @@
         <v>71</v>
       </c>
       <c r="E109" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C109,'feed rations'!$K$8:$K$43,0),MATCH(B109,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>5.7718576563015853</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C109,'feed rations'!$L$8:$L$43,0),MATCH(B109,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>8.277704323848349</v>
       </c>
       <c r="F109" t="s">
         <v>23</v>
@@ -8946,8 +8998,8 @@
         <v>71</v>
       </c>
       <c r="E110" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C110,'feed rations'!$K$8:$K$43,0),MATCH(B110,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>0.60585103137062835</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C110,'feed rations'!$L$8:$L$43,0),MATCH(B110,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>0.86888069675614876</v>
       </c>
       <c r="F110" t="s">
         <v>23</v>
@@ -8964,8 +9016,8 @@
         <v>71</v>
       </c>
       <c r="E111" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C111,'feed rations'!$K$8:$K$43,0),MATCH(B111,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>33.966462264962807</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C111,'feed rations'!$L$8:$L$43,0),MATCH(B111,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>0.16156872460341609</v>
       </c>
       <c r="F111" t="s">
         <v>23</v>
@@ -8982,8 +9034,8 @@
         <v>71</v>
       </c>
       <c r="E112" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C112,'feed rations'!$K$8:$K$43,0),MATCH(B112,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>0</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C112,'feed rations'!$L$8:$L$43,0),MATCH(B112,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>4.6933021685215648</v>
       </c>
       <c r="F112" t="s">
         <v>23</v>
@@ -9000,8 +9052,8 @@
         <v>71</v>
       </c>
       <c r="E113" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C113,'feed rations'!$K$8:$K$43,0),MATCH(B113,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>2.7538683244119473</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C113,'feed rations'!$L$8:$L$43,0),MATCH(B113,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>3.554511941275154</v>
       </c>
       <c r="F113" t="s">
         <v>23</v>
@@ -9018,8 +9070,8 @@
         <v>71</v>
       </c>
       <c r="E114" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C114,'feed rations'!$K$8:$K$43,0),MATCH(B114,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>7.1350224768854983E-2</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C114,'feed rations'!$L$8:$L$43,0),MATCH(B114,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>0.10232685891549684</v>
       </c>
       <c r="F114" t="s">
         <v>23</v>
@@ -9036,8 +9088,8 @@
         <v>71</v>
       </c>
       <c r="E115" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C115,'feed rations'!$K$8:$K$43,0),MATCH(B115,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>2.4545416139233072</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C115,'feed rations'!$L$8:$L$43,0),MATCH(B115,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>4.3583163461771495</v>
       </c>
       <c r="F115" t="s">
         <v>23</v>
@@ -9054,7 +9106,7 @@
         <v>71</v>
       </c>
       <c r="E116" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C116,'feed rations'!$K$8:$K$43,0),MATCH(B116,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C116,'feed rations'!$L$8:$L$43,0),MATCH(B116,'feed rations'!$Q$7:$T$7,0))</f>
         <v>0</v>
       </c>
       <c r="F116" t="s">
@@ -9072,8 +9124,8 @@
         <v>71</v>
       </c>
       <c r="E117" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C117,'feed rations'!$K$8:$K$43,0),MATCH(B117,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>21.826284108458598</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C117,'feed rations'!$L$8:$L$43,0),MATCH(B117,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>31.302145183860713</v>
       </c>
       <c r="F117" t="s">
         <v>23</v>
@@ -9090,8 +9142,8 @@
         <v>71</v>
       </c>
       <c r="E118" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C118,'feed rations'!$K$8:$K$43,0),MATCH(B118,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>16.76667694151628</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C118,'feed rations'!$L$8:$L$43,0),MATCH(B118,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>24.045914241116183</v>
       </c>
       <c r="F118" t="s">
         <v>23</v>
@@ -9108,8 +9160,8 @@
         <v>71</v>
       </c>
       <c r="E119" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C119,'feed rations'!$K$8:$K$43,0),MATCH(B119,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>2.8258444283454405</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C119,'feed rations'!$L$8:$L$43,0),MATCH(B119,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>4.0526821754690197</v>
       </c>
       <c r="F119" t="s">
         <v>23</v>
@@ -9126,8 +9178,8 @@
         <v>71</v>
       </c>
       <c r="E120" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C120,'feed rations'!$K$8:$K$43,0),MATCH(B120,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>2.6374547997890785</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C120,'feed rations'!$L$8:$L$43,0),MATCH(B120,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>3.7825033637710859</v>
       </c>
       <c r="F120" t="s">
         <v>23</v>
@@ -9144,8 +9196,8 @@
         <v>71</v>
       </c>
       <c r="E121" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C121,'feed rations'!$K$8:$K$43,0),MATCH(B121,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>5.3825608158960786E-2</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C121,'feed rations'!$L$8:$L$43,0),MATCH(B121,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>7.7193946199409905E-2</v>
       </c>
       <c r="F121" t="s">
         <v>23</v>
@@ -9162,8 +9214,8 @@
         <v>71</v>
       </c>
       <c r="E122" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C122,'feed rations'!$K$8:$K$43,0),MATCH(B122,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>0.31919837396593026</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C122,'feed rations'!$L$8:$L$43,0),MATCH(B122,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>0.45777805304301217</v>
       </c>
       <c r="F122" t="s">
         <v>23</v>
@@ -9180,8 +9232,8 @@
         <v>71</v>
       </c>
       <c r="E123" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C123,'feed rations'!$K$8:$K$43,0),MATCH(B123,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>5.3997724929236526</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C123,'feed rations'!$L$8:$L$43,0),MATCH(B123,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>7.74407873064429</v>
       </c>
       <c r="F123" t="s">
         <v>23</v>
@@ -9198,8 +9250,8 @@
         <v>71</v>
       </c>
       <c r="E124" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C124,'feed rations'!$K$8:$K$43,0),MATCH(B124,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>1.9827851935766017</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C124,'feed rations'!$L$8:$L$43,0),MATCH(B124,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>2.8436095530201233</v>
       </c>
       <c r="F124" t="s">
         <v>23</v>
@@ -9216,8 +9268,8 @@
         <v>71</v>
       </c>
       <c r="E125" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C125,'feed rations'!$K$8:$K$43,0),MATCH(B125,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>2.4503169295619931</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C125,'feed rations'!$L$8:$L$43,0),MATCH(B125,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>3.5141197601242991</v>
       </c>
       <c r="F125" t="s">
         <v>23</v>
@@ -9234,8 +9286,8 @@
         <v>71</v>
       </c>
       <c r="E126" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C126,'feed rations'!$K$8:$K$43,0),MATCH(B126,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>0.11391000796431236</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C126,'feed rations'!$L$8:$L$43,0),MATCH(B126,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>0.16336393265456514</v>
       </c>
       <c r="F126" t="s">
         <v>23</v>
@@ -9252,8 +9304,8 @@
         <v>71</v>
       </c>
       <c r="E127" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C127,'feed rations'!$K$8:$K$43,0),MATCH(B127,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>5.7718576563015853</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C127,'feed rations'!$L$8:$L$43,0),MATCH(B127,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>8.277704323848349</v>
       </c>
       <c r="F127" t="s">
         <v>23</v>
@@ -9270,8 +9322,8 @@
         <v>71</v>
       </c>
       <c r="E128" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C128,'feed rations'!$K$8:$K$43,0),MATCH(B128,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>0.60585103137062835</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C128,'feed rations'!$L$8:$L$43,0),MATCH(B128,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>0.86888069675614876</v>
       </c>
       <c r="F128" t="s">
         <v>23</v>
@@ -9288,8 +9340,8 @@
         <v>71</v>
       </c>
       <c r="E129" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C129,'feed rations'!$K$8:$K$43,0),MATCH(B129,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>33.966462264962807</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C129,'feed rations'!$L$8:$L$43,0),MATCH(B129,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>0.16156872460341609</v>
       </c>
       <c r="F129" t="s">
         <v>23</v>
@@ -9306,8 +9358,8 @@
         <v>71</v>
       </c>
       <c r="E130" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C130,'feed rations'!$K$8:$K$43,0),MATCH(B130,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>0</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C130,'feed rations'!$L$8:$L$43,0),MATCH(B130,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>4.6933021685215648</v>
       </c>
       <c r="F130" t="s">
         <v>23</v>
@@ -9324,8 +9376,8 @@
         <v>71</v>
       </c>
       <c r="E131" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C131,'feed rations'!$K$8:$K$43,0),MATCH(B131,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>2.7538683244119473</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C131,'feed rations'!$L$8:$L$43,0),MATCH(B131,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>3.554511941275154</v>
       </c>
       <c r="F131" t="s">
         <v>23</v>
@@ -9342,8 +9394,8 @@
         <v>71</v>
       </c>
       <c r="E132" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C132,'feed rations'!$K$8:$K$43,0),MATCH(B132,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>7.1350224768854983E-2</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C132,'feed rations'!$L$8:$L$43,0),MATCH(B132,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>0.10232685891549684</v>
       </c>
       <c r="F132" t="s">
         <v>23</v>
@@ -9360,8 +9412,8 @@
         <v>71</v>
       </c>
       <c r="E133" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C133,'feed rations'!$K$8:$K$43,0),MATCH(B133,'feed rations'!$Q$7:$T$7,0))</f>
-        <v>2.4545416139233072</v>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C133,'feed rations'!$L$8:$L$43,0),MATCH(B133,'feed rations'!$Q$7:$T$7,0))</f>
+        <v>4.3583163461771495</v>
       </c>
       <c r="F133" t="s">
         <v>23</v>
@@ -9378,7 +9430,7 @@
         <v>71</v>
       </c>
       <c r="E134" s="62">
-        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C134,'feed rations'!$K$8:$K$43,0),MATCH(B134,'feed rations'!$Q$7:$T$7,0))</f>
+        <f>INDEX('feed rations'!$Q$8:$T$43,MATCH(C134,'feed rations'!$L$8:$L$43,0),MATCH(B134,'feed rations'!$Q$7:$T$7,0))</f>
         <v>0</v>
       </c>
       <c r="F134" t="s">
@@ -9392,7 +9444,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A5:Z50"/>
+  <dimension ref="A5:V52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -9403,8 +9455,9 @@
     <col min="7" max="7" width="4.85546875" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
     <col min="9" max="9" width="5.42578125" customWidth="1"/>
-    <col min="11" max="11" width="27.7109375" customWidth="1"/>
-    <col min="12" max="14" width="13.28515625" customWidth="1"/>
+    <col min="10" max="10" width="8.28515625" customWidth="1"/>
+    <col min="12" max="12" width="27.7109375" customWidth="1"/>
+    <col min="13" max="15" width="13.28515625" customWidth="1"/>
     <col min="17" max="20" width="10.28515625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -9425,69 +9478,67 @@
       <c r="G6" s="105"/>
       <c r="H6" s="105"/>
       <c r="I6" s="106"/>
-      <c r="L6" s="90" t="s">
-        <v>248</v>
-      </c>
-      <c r="O6" s="78"/>
+      <c r="J6" s="112"/>
+      <c r="M6" s="90" t="s">
+        <v>238</v>
+      </c>
       <c r="Q6" s="90" t="s">
-        <v>249</v>
+        <v>239</v>
       </c>
     </row>
     <row r="7" spans="2:22" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
         <v>210</v>
       </c>
-      <c r="C7" s="115"/>
-      <c r="D7" s="131" t="s">
+      <c r="C7" s="114"/>
+      <c r="D7" s="127" t="s">
         <v>169</v>
       </c>
-      <c r="E7" s="131" t="s">
+      <c r="E7" s="127" t="s">
         <v>23</v>
       </c>
-      <c r="F7" s="131" t="s">
+      <c r="F7" s="127" t="s">
         <v>170</v>
       </c>
-      <c r="G7" s="131" t="s">
+      <c r="G7" s="127" t="s">
         <v>23</v>
       </c>
-      <c r="H7" s="131" t="s">
+      <c r="H7" s="127" t="s">
         <v>171</v>
       </c>
-      <c r="I7" s="132" t="s">
+      <c r="I7" s="128" t="s">
         <v>23</v>
       </c>
-      <c r="K7" s="91" t="s">
+      <c r="J7" s="135" t="s">
+        <v>209</v>
+      </c>
+      <c r="L7" s="91" t="s">
         <v>210</v>
       </c>
-      <c r="L7" s="129" t="s">
+      <c r="M7" s="125" t="s">
+        <v>230</v>
+      </c>
+      <c r="N7" s="131" t="s">
+        <v>15</v>
+      </c>
+      <c r="O7" s="126" t="s">
         <v>240</v>
       </c>
-      <c r="M7" s="135" t="s">
+      <c r="P7" s="91"/>
+      <c r="Q7" s="125">
+        <v>0</v>
+      </c>
+      <c r="R7" s="131" t="s">
         <v>15</v>
       </c>
-      <c r="N7" s="130" t="s">
-        <v>250</v>
-      </c>
-      <c r="O7" s="139" t="s">
-        <v>209</v>
-      </c>
-      <c r="P7" s="91"/>
-      <c r="Q7" s="129">
-        <v>0</v>
-      </c>
-      <c r="R7" s="135" t="s">
-        <v>15</v>
-      </c>
-      <c r="S7" s="135" t="s">
+      <c r="S7" s="131" t="s">
         <v>24</v>
       </c>
-      <c r="T7" s="130" t="s">
+      <c r="T7" s="126" t="s">
         <v>25</v>
       </c>
       <c r="U7" s="108"/>
-      <c r="V7" s="92" t="s">
-        <v>232</v>
-      </c>
+      <c r="V7" s="92"/>
     </row>
     <row r="8" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
@@ -9517,39 +9568,39 @@
         <f t="shared" ref="I8:I42" si="2">H8/H$45</f>
         <v>0.15836750634641669</v>
       </c>
-      <c r="K8" t="s">
+      <c r="J8" s="136">
+        <v>86</v>
+      </c>
+      <c r="L8" t="s">
         <v>70</v>
       </c>
-      <c r="L8" s="97">
-        <f>(D8)*($O8/100)</f>
+      <c r="M8" s="97">
+        <f>D8*($J8/100)</f>
         <v>445.13600000000002</v>
       </c>
-      <c r="M8" s="99">
-        <f>(F8)*($O8/100)</f>
+      <c r="N8" s="99">
+        <f>F8*($J8/100)</f>
         <v>12.814</v>
       </c>
-      <c r="N8" s="134">
-        <f>(H8)*($O8/100)</f>
+      <c r="O8" s="130">
+        <f>H8*($J8/100)</f>
         <v>69.745999999999995</v>
       </c>
-      <c r="O8" s="140">
-        <v>86</v>
-      </c>
-      <c r="Q8" s="136">
-        <f t="shared" ref="Q8:Q33" si="3">L8/L$44*100</f>
+      <c r="Q8" s="132">
+        <f>M8/M$44*100</f>
         <v>39.939446969082496</v>
       </c>
       <c r="R8" s="98">
-        <f t="shared" ref="R8:R33" si="4">M8/M$44*100</f>
+        <f>N8/N$44*100</f>
         <v>37.344664381805039</v>
       </c>
-      <c r="S8" s="138">
-        <f t="shared" ref="S8:S33" si="5">N8/N$44*100</f>
-        <v>21.826284108458598</v>
+      <c r="S8" s="134">
+        <f>O8/O$44*100</f>
+        <v>31.302145183860713</v>
       </c>
       <c r="T8" s="102">
-        <f>N8/N$44*100</f>
-        <v>21.826284108458598</v>
+        <f>O8/O$44*100</f>
+        <v>31.302145183860713</v>
       </c>
       <c r="U8" s="98"/>
     </row>
@@ -9581,39 +9632,39 @@
         <f t="shared" si="2"/>
         <v>0.12165592657684045</v>
       </c>
-      <c r="K9" t="s">
+      <c r="J9" s="136">
+        <v>86</v>
+      </c>
+      <c r="L9" t="s">
         <v>160</v>
       </c>
-      <c r="L9" s="97">
-        <f>(D9)*($O9/100)</f>
+      <c r="M9" s="97">
+        <f>D9*($J9/100)</f>
         <v>374.358</v>
       </c>
-      <c r="M9" s="99">
-        <f>(F9)*($O9/100)</f>
+      <c r="N9" s="99">
+        <f>F9*($J9/100)</f>
         <v>11.61</v>
       </c>
-      <c r="N9" s="134">
-        <f>(H9)*($O9/100)</f>
+      <c r="O9" s="130">
+        <f>H9*($J9/100)</f>
         <v>53.577999999999996</v>
       </c>
-      <c r="O9" s="140">
-        <v>86</v>
-      </c>
-      <c r="Q9" s="136">
-        <f t="shared" si="3"/>
+      <c r="Q9" s="132">
+        <f>M9/M$44*100</f>
         <v>33.588951440574981</v>
       </c>
       <c r="R9" s="98">
-        <f t="shared" si="4"/>
+        <f>N9/N$44*100</f>
         <v>33.835769741903896</v>
       </c>
       <c r="S9" s="98">
-        <f t="shared" si="5"/>
-        <v>16.76667694151628</v>
+        <f>O9/O$44*100</f>
+        <v>24.045914241116183</v>
       </c>
       <c r="T9" s="102">
-        <f t="shared" ref="T9:T33" si="6">N9/N$44*100</f>
-        <v>16.76667694151628</v>
+        <f>O9/O$44*100</f>
+        <v>24.045914241116183</v>
       </c>
       <c r="U9" s="98"/>
     </row>
@@ -9645,39 +9696,39 @@
         <f t="shared" si="2"/>
         <v>2.0503807850029289E-2</v>
       </c>
-      <c r="K10" t="s">
+      <c r="J10" s="136">
+        <v>86</v>
+      </c>
+      <c r="L10" t="s">
         <v>161</v>
       </c>
-      <c r="L10" s="97">
-        <f>(D10+D36)*($O10/100)</f>
+      <c r="M10" s="97">
+        <f>D10*($J10/100)+D36*($J36/100)</f>
         <v>54.352000000000004</v>
       </c>
-      <c r="M10" s="99">
-        <f>(F10+F36)*($O10/100)</f>
+      <c r="N10" s="99">
+        <f>F10*($J10/100)+F36*($J36/100)</f>
         <v>2.4940000000000002</v>
       </c>
-      <c r="N10" s="134">
-        <f>(H10+H36)*($O10/100)</f>
+      <c r="O10" s="130">
+        <f>H10*($J10/100)+H36*($J36/100)</f>
         <v>9.0299999999999994</v>
       </c>
-      <c r="O10" s="140">
-        <v>86</v>
-      </c>
-      <c r="Q10" s="136">
-        <f t="shared" si="3"/>
+      <c r="Q10" s="132">
+        <f>M10/M$44*100</f>
         <v>4.876686724200181</v>
       </c>
       <c r="R10" s="98">
-        <f t="shared" si="4"/>
+        <f>N10/N$44*100</f>
         <v>7.2684246112238</v>
       </c>
       <c r="S10" s="98">
-        <f t="shared" si="5"/>
-        <v>2.8258444283454405</v>
+        <f>O10/O$44*100</f>
+        <v>4.0526821754690197</v>
       </c>
       <c r="T10" s="102">
-        <f t="shared" si="6"/>
-        <v>2.8258444283454405</v>
+        <f>O10/O$44*100</f>
+        <v>4.0526821754690197</v>
       </c>
       <c r="U10" s="98"/>
     </row>
@@ -9709,39 +9760,39 @@
         <f t="shared" si="2"/>
         <v>1.9136887326694007E-2</v>
       </c>
-      <c r="K11" t="s">
+      <c r="J11" s="136">
+        <v>86</v>
+      </c>
+      <c r="L11" t="s">
         <v>162</v>
       </c>
-      <c r="L11" s="97">
-        <f t="shared" ref="L11:L21" si="7">(D11)*($O11/100)</f>
+      <c r="M11" s="97">
+        <f>D11*($J11/100)</f>
         <v>4.9879999999999995</v>
       </c>
-      <c r="M11" s="99">
-        <f t="shared" ref="M11:M21" si="8">(F11)*($O11/100)</f>
-        <v>0</v>
-      </c>
-      <c r="N11" s="134">
-        <f t="shared" ref="N11:N21" si="9">(H11)*($O11/100)</f>
+      <c r="N11" s="99">
+        <f>F11*($J11/100)</f>
+        <v>0</v>
+      </c>
+      <c r="O11" s="130">
+        <f>H11*($J11/100)</f>
         <v>8.4280000000000008</v>
       </c>
-      <c r="O11" s="140">
-        <v>86</v>
-      </c>
-      <c r="Q11" s="136">
-        <f t="shared" si="3"/>
+      <c r="Q11" s="132">
+        <f>M11/M$44*100</f>
         <v>0.44754403481583932</v>
       </c>
       <c r="R11" s="98">
-        <f t="shared" si="4"/>
+        <f>N11/N$44*100</f>
         <v>0</v>
       </c>
       <c r="S11" s="98">
-        <f t="shared" si="5"/>
-        <v>2.6374547997890785</v>
+        <f>O11/O$44*100</f>
+        <v>3.7825033637710859</v>
       </c>
       <c r="T11" s="102">
-        <f t="shared" si="6"/>
-        <v>2.6374547997890785</v>
+        <f>O11/O$44*100</f>
+        <v>3.7825033637710859</v>
       </c>
       <c r="U11" s="98"/>
     </row>
@@ -9773,39 +9824,39 @@
         <f t="shared" si="2"/>
         <v>3.905487209529389E-4</v>
       </c>
-      <c r="K12" t="s">
+      <c r="J12" s="136">
+        <v>86</v>
+      </c>
+      <c r="L12" t="s">
         <v>165</v>
       </c>
-      <c r="L12" s="97">
-        <f t="shared" si="7"/>
+      <c r="M12" s="97">
+        <f>D12*($J12/100)</f>
         <v>2.4939999999999998</v>
       </c>
-      <c r="M12" s="99">
-        <f t="shared" si="8"/>
+      <c r="N12" s="99">
+        <f>F12*($J12/100)</f>
         <v>0.60199999999999998</v>
       </c>
-      <c r="N12" s="134">
-        <f t="shared" si="9"/>
+      <c r="O12" s="130">
+        <f>H12*($J12/100)</f>
         <v>0.17200000000000001</v>
       </c>
-      <c r="O12" s="140">
-        <v>86</v>
-      </c>
-      <c r="Q12" s="136">
-        <f t="shared" si="3"/>
+      <c r="Q12" s="132">
+        <f>M12/M$44*100</f>
         <v>0.22377201740791966</v>
       </c>
       <c r="R12" s="98">
-        <f t="shared" si="4"/>
+        <f>N12/N$44*100</f>
         <v>1.7544473199505721</v>
       </c>
       <c r="S12" s="98">
-        <f t="shared" si="5"/>
-        <v>5.3825608158960786E-2</v>
+        <f>O12/O$44*100</f>
+        <v>7.7193946199409905E-2</v>
       </c>
       <c r="T12" s="102">
-        <f t="shared" si="6"/>
-        <v>5.3825608158960786E-2</v>
+        <f>O12/O$44*100</f>
+        <v>7.7193946199409905E-2</v>
       </c>
       <c r="U12" s="98"/>
     </row>
@@ -9837,39 +9888,39 @@
         <f t="shared" si="2"/>
         <v>2.3432923257176333E-3</v>
       </c>
-      <c r="K13" t="s">
+      <c r="J13" s="136">
+        <v>85</v>
+      </c>
+      <c r="L13" t="s">
         <v>218</v>
       </c>
-      <c r="L13" s="97">
-        <f t="shared" si="7"/>
+      <c r="M13" s="97">
+        <f>D13*($J13/100)</f>
         <v>8.7550000000000008</v>
       </c>
-      <c r="M13" s="99">
-        <f t="shared" si="8"/>
+      <c r="N13" s="99">
+        <f>F13*($J13/100)</f>
         <v>8.5000000000000006E-2</v>
       </c>
-      <c r="N13" s="134">
-        <f t="shared" si="9"/>
+      <c r="O13" s="130">
+        <f>H13*($J13/100)</f>
         <v>1.02</v>
       </c>
-      <c r="O13" s="140">
-        <v>85</v>
-      </c>
-      <c r="Q13" s="136">
-        <f t="shared" si="3"/>
+      <c r="Q13" s="132">
+        <f>M13/M$44*100</f>
         <v>0.78553488869540378</v>
       </c>
       <c r="R13" s="98">
-        <f t="shared" si="4"/>
+        <f>N13/N$44*100</f>
         <v>0.24772096710265556</v>
       </c>
       <c r="S13" s="98">
-        <f t="shared" si="5"/>
-        <v>0.31919837396593026</v>
+        <f>O13/O$44*100</f>
+        <v>0.45777805304301217</v>
       </c>
       <c r="T13" s="102">
-        <f t="shared" si="6"/>
-        <v>0.31919837396593026</v>
+        <f>O13/O$44*100</f>
+        <v>0.45777805304301217</v>
       </c>
       <c r="U13" s="98"/>
     </row>
@@ -9901,39 +9952,39 @@
         <f t="shared" si="2"/>
         <v>3.9640695176723299E-2</v>
       </c>
-      <c r="K14" t="s">
+      <c r="J14" s="136">
+        <v>85</v>
+      </c>
+      <c r="L14" t="s">
         <v>219</v>
       </c>
-      <c r="L14" s="97">
-        <f t="shared" si="7"/>
+      <c r="M14" s="97">
+        <f>D14*($J14/100)</f>
         <v>1.105</v>
       </c>
-      <c r="M14" s="99">
-        <f t="shared" si="8"/>
+      <c r="N14" s="99">
+        <f>F14*($J14/100)</f>
         <v>0.255</v>
       </c>
-      <c r="N14" s="134">
-        <f t="shared" si="9"/>
+      <c r="O14" s="130">
+        <f>H14*($J14/100)</f>
         <v>17.254999999999999</v>
       </c>
-      <c r="O14" s="140">
-        <v>85</v>
-      </c>
-      <c r="Q14" s="136">
-        <f t="shared" si="3"/>
+      <c r="Q14" s="132">
+        <f>M14/M$44*100</f>
         <v>9.9145180126604351E-2</v>
       </c>
       <c r="R14" s="98">
-        <f t="shared" si="4"/>
+        <f>N14/N$44*100</f>
         <v>0.74316290130796658</v>
       </c>
       <c r="S14" s="98">
-        <f t="shared" si="5"/>
-        <v>5.3997724929236526</v>
+        <f>O14/O$44*100</f>
+        <v>7.74407873064429</v>
       </c>
       <c r="T14" s="102">
-        <f t="shared" si="6"/>
-        <v>5.3997724929236526</v>
+        <f>O14/O$44*100</f>
+        <v>7.74407873064429</v>
       </c>
       <c r="U14" s="98"/>
     </row>
@@ -9965,38 +10016,38 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="K15" t="s">
+      <c r="J15" s="136">
+        <v>91</v>
+      </c>
+      <c r="L15" t="s">
         <v>163</v>
       </c>
-      <c r="L15" s="97">
-        <f t="shared" si="7"/>
+      <c r="M15" s="97">
+        <f>D15*($J15/100)</f>
         <v>3.9129999999999998</v>
       </c>
-      <c r="M15" s="99">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="N15" s="134">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="O15" s="140">
-        <v>91</v>
-      </c>
-      <c r="Q15" s="136">
-        <f t="shared" si="3"/>
+      <c r="N15" s="99">
+        <f>F15*($J15/100)</f>
+        <v>0</v>
+      </c>
+      <c r="O15" s="130">
+        <f>H15*($J15/100)</f>
+        <v>0</v>
+      </c>
+      <c r="Q15" s="132">
+        <f>M15/M$44*100</f>
         <v>0.35109057903656365</v>
       </c>
       <c r="R15" s="98">
-        <f t="shared" si="4"/>
+        <f>N15/N$44*100</f>
         <v>0</v>
       </c>
       <c r="S15" s="98">
-        <f t="shared" si="5"/>
+        <f>O15/O$44*100</f>
         <v>0</v>
       </c>
       <c r="T15" s="102">
-        <f t="shared" si="6"/>
+        <f>O15/O$44*100</f>
         <v>0</v>
       </c>
       <c r="U15" s="98"/>
@@ -10029,43 +10080,43 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="K16" t="s">
+      <c r="J16" s="136">
+        <v>91</v>
+      </c>
+      <c r="L16" t="s">
         <v>164</v>
       </c>
-      <c r="L16" s="97">
-        <f t="shared" si="7"/>
+      <c r="M16" s="97">
+        <f>D16*($J16/100)</f>
         <v>1.4560000000000002</v>
       </c>
-      <c r="M16" s="99">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="N16" s="134">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="O16" s="140">
-        <v>91</v>
-      </c>
-      <c r="Q16" s="136">
-        <f t="shared" si="3"/>
+      <c r="N16" s="99">
+        <f>F16*($J16/100)</f>
+        <v>0</v>
+      </c>
+      <c r="O16" s="130">
+        <f>H16*($J16/100)</f>
+        <v>0</v>
+      </c>
+      <c r="Q16" s="132">
+        <f>M16/M$44*100</f>
         <v>0.13063835499034929</v>
       </c>
       <c r="R16" s="98">
-        <f t="shared" si="4"/>
+        <f>N16/N$44*100</f>
         <v>0</v>
       </c>
       <c r="S16" s="98">
-        <f t="shared" si="5"/>
+        <f>O16/O$44*100</f>
         <v>0</v>
       </c>
       <c r="T16" s="102">
-        <f t="shared" si="6"/>
+        <f>O16/O$44*100</f>
         <v>0</v>
       </c>
       <c r="U16" s="98"/>
     </row>
-    <row r="17" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>220</v>
       </c>
@@ -10093,43 +10144,43 @@
         <f t="shared" si="2"/>
         <v>1.4059753954305799E-2</v>
       </c>
-      <c r="K17" t="s">
+      <c r="J17" s="136">
+        <v>88</v>
+      </c>
+      <c r="L17" t="s">
         <v>220</v>
       </c>
-      <c r="L17" s="97">
-        <f t="shared" si="7"/>
+      <c r="M17" s="97">
+        <f>D17*($J17/100)</f>
         <v>77.967999999999989</v>
       </c>
-      <c r="M17" s="99">
-        <f t="shared" si="8"/>
+      <c r="N17" s="99">
+        <f>F17*($J17/100)</f>
         <v>2.464</v>
       </c>
-      <c r="N17" s="134">
-        <f t="shared" si="9"/>
+      <c r="O17" s="130">
+        <f>H17*($J17/100)</f>
         <v>6.3360000000000003</v>
       </c>
-      <c r="O17" s="140">
-        <v>88</v>
-      </c>
-      <c r="Q17" s="136">
-        <f t="shared" si="3"/>
+      <c r="Q17" s="132">
+        <f>M17/M$44*100</f>
         <v>6.9956121304172738</v>
       </c>
       <c r="R17" s="98">
-        <f t="shared" si="4"/>
+        <f>N17/N$44*100</f>
         <v>7.1809936816581557</v>
       </c>
       <c r="S17" s="98">
-        <f t="shared" si="5"/>
-        <v>1.9827851935766017</v>
+        <f>O17/O$44*100</f>
+        <v>2.8436095530201233</v>
       </c>
       <c r="T17" s="102">
-        <f t="shared" si="6"/>
-        <v>1.9827851935766017</v>
+        <f>O17/O$44*100</f>
+        <v>2.8436095530201233</v>
       </c>
       <c r="U17" s="98"/>
     </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
         <v>222</v>
       </c>
@@ -10157,46 +10208,43 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="K18" t="s">
+      <c r="J18" s="136">
+        <v>87</v>
+      </c>
+      <c r="L18" t="s">
         <v>222</v>
       </c>
-      <c r="L18" s="97">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="M18" s="99">
-        <f t="shared" si="8"/>
+      <c r="M18" s="97">
+        <f>D18*($J18/100)</f>
+        <v>0</v>
+      </c>
+      <c r="N18" s="99">
+        <f>F18*($J18/100)</f>
         <v>0.78300000000000003</v>
       </c>
-      <c r="N18" s="134">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="O18" s="140">
-        <v>87</v>
-      </c>
-      <c r="Q18" s="136">
-        <f t="shared" si="3"/>
+      <c r="O18" s="130">
+        <f>H18*($J18/100)</f>
+        <v>0</v>
+      </c>
+      <c r="Q18" s="132">
+        <f>M18/M$44*100</f>
         <v>0</v>
       </c>
       <c r="R18" s="98">
-        <f t="shared" si="4"/>
+        <f>N18/N$44*100</f>
         <v>2.2819472616632859</v>
       </c>
       <c r="S18" s="98">
-        <f t="shared" si="5"/>
+        <f>O18/O$44*100</f>
         <v>0</v>
       </c>
       <c r="T18" s="102">
-        <f t="shared" si="6"/>
+        <f>O18/O$44*100</f>
         <v>0</v>
       </c>
       <c r="U18" s="98"/>
-      <c r="V18" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="19" spans="1:26" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>221</v>
       </c>
@@ -10224,46 +10272,43 @@
         <f t="shared" si="2"/>
         <v>1.698886936145284E-2</v>
       </c>
-      <c r="K19" t="s">
+      <c r="J19" s="136">
+        <v>90</v>
+      </c>
+      <c r="L19" t="s">
         <v>221</v>
       </c>
-      <c r="L19" s="97">
-        <f t="shared" si="7"/>
+      <c r="M19" s="97">
+        <f>D19*($J19/100)</f>
         <v>36.630000000000003</v>
       </c>
-      <c r="M19" s="99">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="N19" s="134">
-        <f t="shared" si="9"/>
+      <c r="N19" s="99">
+        <f>F19*($J19/100)</f>
+        <v>0</v>
+      </c>
+      <c r="O19" s="130">
+        <f>H19*($J19/100)</f>
         <v>7.8299999999999992</v>
       </c>
-      <c r="O19" s="140">
-        <v>90</v>
-      </c>
-      <c r="Q19" s="136">
-        <f t="shared" si="3"/>
+      <c r="Q19" s="132">
+        <f>M19/M$44*100</f>
         <v>3.2865954280882512</v>
       </c>
       <c r="R19" s="98">
-        <f t="shared" si="4"/>
+        <f>N19/N$44*100</f>
         <v>0</v>
       </c>
       <c r="S19" s="98">
-        <f t="shared" si="5"/>
-        <v>2.4503169295619931</v>
+        <f>O19/O$44*100</f>
+        <v>3.5141197601242991</v>
       </c>
       <c r="T19" s="102">
-        <f t="shared" si="6"/>
-        <v>2.4503169295619931</v>
+        <f>O19/O$44*100</f>
+        <v>3.5141197601242991</v>
       </c>
       <c r="U19" s="98"/>
-      <c r="V19" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="20" spans="1:26" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B20" t="s">
         <v>217</v>
       </c>
@@ -10291,43 +10336,43 @@
         <f t="shared" si="2"/>
         <v>7.810974419058778E-4</v>
       </c>
-      <c r="K20" t="s">
+      <c r="J20" s="136">
+        <v>91</v>
+      </c>
+      <c r="L20" t="s">
         <v>217</v>
       </c>
-      <c r="L20" s="97">
-        <f t="shared" si="7"/>
+      <c r="M20" s="97">
+        <f>D20*($J20/100)</f>
         <v>5.0049999999999999</v>
       </c>
-      <c r="M20" s="99">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="N20" s="134">
-        <f t="shared" si="9"/>
+      <c r="N20" s="99">
+        <f>F20*($J20/100)</f>
+        <v>0</v>
+      </c>
+      <c r="O20" s="130">
+        <f>H20*($J20/100)</f>
         <v>0.36400000000000005</v>
       </c>
-      <c r="O20" s="140">
-        <v>91</v>
-      </c>
-      <c r="Q20" s="136">
-        <f t="shared" si="3"/>
+      <c r="Q20" s="132">
+        <f>M20/M$44*100</f>
         <v>0.44906934527932563</v>
       </c>
       <c r="R20" s="98">
-        <f t="shared" si="4"/>
+        <f>N20/N$44*100</f>
         <v>0</v>
       </c>
       <c r="S20" s="98">
-        <f t="shared" si="5"/>
-        <v>0.11391000796431236</v>
+        <f>O20/O$44*100</f>
+        <v>0.16336393265456514</v>
       </c>
       <c r="T20" s="102">
-        <f t="shared" si="6"/>
-        <v>0.11391000796431236</v>
+        <f>O20/O$44*100</f>
+        <v>0.16336393265456514</v>
       </c>
       <c r="U20" s="98"/>
     </row>
-    <row r="21" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
         <v>213</v>
       </c>
@@ -10355,46 +10400,43 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="K21" t="s">
+      <c r="J21" s="136">
+        <v>91</v>
+      </c>
+      <c r="L21" t="s">
         <v>213</v>
       </c>
-      <c r="L21" s="97">
-        <f t="shared" si="7"/>
+      <c r="M21" s="97">
+        <f>D21*($J21/100)</f>
         <v>1.4560000000000002</v>
       </c>
-      <c r="M21" s="99">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="N21" s="134">
-        <f t="shared" si="9"/>
-        <v>0</v>
-      </c>
-      <c r="O21" s="140">
-        <v>91</v>
-      </c>
-      <c r="Q21" s="136">
-        <f t="shared" si="3"/>
+      <c r="N21" s="99">
+        <f>F21*($J21/100)</f>
+        <v>0</v>
+      </c>
+      <c r="O21" s="130">
+        <f>H21*($J21/100)</f>
+        <v>0</v>
+      </c>
+      <c r="Q21" s="132">
+        <f>M21/M$44*100</f>
         <v>0.13063835499034929</v>
       </c>
       <c r="R21" s="98">
-        <f t="shared" si="4"/>
+        <f>N21/N$44*100</f>
         <v>0</v>
       </c>
       <c r="S21" s="98">
-        <f t="shared" si="5"/>
+        <f>O21/O$44*100</f>
         <v>0</v>
       </c>
       <c r="T21" s="102">
-        <f t="shared" si="6"/>
+        <f>O21/O$44*100</f>
         <v>0</v>
       </c>
       <c r="U21" s="98"/>
-      <c r="V21" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="22" spans="1:26" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>214</v>
       </c>
@@ -10422,43 +10464,43 @@
         <f t="shared" si="2"/>
         <v>6.444053895723491E-3</v>
       </c>
-      <c r="K22" t="s">
+      <c r="J22" s="136">
+        <v>87</v>
+      </c>
+      <c r="L22" t="s">
         <v>214</v>
       </c>
-      <c r="L22" s="97">
-        <f>(D22+D39)*($O22/100)</f>
+      <c r="M22" s="97">
+        <f>D22*($J22/100)+D39*($J39/100)</f>
         <v>34.713000000000001</v>
       </c>
-      <c r="M22" s="99">
-        <f>(F22+F39)*($O22/100)</f>
-        <v>0</v>
-      </c>
-      <c r="N22" s="134">
-        <f>(H22+H39)*($O22/100)</f>
+      <c r="N22" s="99">
+        <f>F22*($J22/100)+F39*($J39/100)</f>
+        <v>0</v>
+      </c>
+      <c r="O22" s="130">
+        <f>H22*($J22/100)+H39*($J39/100)</f>
         <v>18.443999999999999</v>
       </c>
-      <c r="O22" s="140">
-        <v>87</v>
-      </c>
-      <c r="Q22" s="136">
-        <f t="shared" si="3"/>
+      <c r="Q22" s="132">
+        <f>M22/M$44*100</f>
         <v>3.1145942422939523</v>
       </c>
       <c r="R22" s="98">
-        <f t="shared" si="4"/>
+        <f>N22/N$44*100</f>
         <v>0</v>
       </c>
       <c r="S22" s="98">
-        <f t="shared" si="5"/>
-        <v>5.7718576563015853</v>
+        <f>O22/O$44*100</f>
+        <v>8.277704323848349</v>
       </c>
       <c r="T22" s="102">
-        <f t="shared" si="6"/>
-        <v>5.7718576563015853</v>
+        <f>O22/O$44*100</f>
+        <v>8.277704323848349</v>
       </c>
       <c r="U22" s="98"/>
     </row>
-    <row r="23" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="87" t="s">
         <v>215</v>
       </c>
@@ -10489,43 +10531,43 @@
         <f t="shared" si="2"/>
         <v>4.2960359304823276E-3</v>
       </c>
-      <c r="K23" t="s">
+      <c r="J23" s="136">
+        <v>88</v>
+      </c>
+      <c r="L23" t="s">
         <v>216</v>
       </c>
-      <c r="L23" s="97">
-        <f>(D23)*($O23/100)</f>
+      <c r="M23" s="97">
+        <f>D23*($J23/100)</f>
         <v>26.135999999999999</v>
       </c>
-      <c r="M23" s="99">
-        <f>(F23)*($O23/100)</f>
+      <c r="N23" s="99">
+        <f>F23*($J23/100)</f>
         <v>0.44</v>
       </c>
-      <c r="N23" s="134">
-        <f>(H23)*($O23/100)</f>
+      <c r="O23" s="130">
+        <f>H23*($J23/100)</f>
         <v>1.9360000000000002</v>
       </c>
-      <c r="O23" s="140">
-        <v>88</v>
-      </c>
-      <c r="Q23" s="136">
-        <f t="shared" si="3"/>
+      <c r="Q23" s="132">
+        <f>M23/M$44*100</f>
         <v>2.3450302513926982</v>
       </c>
       <c r="R23" s="98">
-        <f t="shared" si="4"/>
+        <f>N23/N$44*100</f>
         <v>1.2823203002960992</v>
       </c>
       <c r="S23" s="98">
-        <f t="shared" si="5"/>
-        <v>0.60585103137062835</v>
+        <f>O23/O$44*100</f>
+        <v>0.86888069675614876</v>
       </c>
       <c r="T23" s="102">
-        <f t="shared" si="6"/>
-        <v>0.60585103137062835</v>
+        <f>O23/O$44*100</f>
+        <v>0.86888069675614876</v>
       </c>
       <c r="U23" s="98"/>
     </row>
-    <row r="24" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
         <v>225</v>
       </c>
@@ -10553,43 +10595,43 @@
         <f t="shared" si="2"/>
         <v>7.810974419058778E-4</v>
       </c>
-      <c r="K24" t="s">
+      <c r="J24" s="136">
+        <v>90</v>
+      </c>
+      <c r="L24" t="s">
         <v>225</v>
       </c>
-      <c r="L24" s="97">
-        <f>(D24+D37)*($O24/100)</f>
+      <c r="M24" s="97">
+        <f>D24*($J24/100)</f>
         <v>1.53</v>
       </c>
-      <c r="M24" s="99">
-        <f>(F24+F37)*($O24/100)</f>
-        <v>0</v>
-      </c>
-      <c r="N24" s="134">
-        <f>(H24+H37)*($O24/100)</f>
-        <v>108.54</v>
-      </c>
-      <c r="O24" s="140">
-        <v>90</v>
-      </c>
-      <c r="Q24" s="136">
-        <f t="shared" si="3"/>
+      <c r="N24" s="99">
+        <f>F24*($J24/100)</f>
+        <v>0</v>
+      </c>
+      <c r="O24" s="130">
+        <f>H24*($J24/100)</f>
+        <v>0.36000000000000004</v>
+      </c>
+      <c r="Q24" s="132">
+        <f>M24/M$44*100</f>
         <v>0.13727794171375987</v>
       </c>
       <c r="R24" s="98">
-        <f t="shared" si="4"/>
+        <f>N24/N$44*100</f>
         <v>0</v>
       </c>
       <c r="S24" s="98">
-        <f t="shared" si="5"/>
-        <v>33.966462264962807</v>
+        <f>O24/O$44*100</f>
+        <v>0.16156872460341609</v>
       </c>
       <c r="T24" s="102">
-        <f t="shared" si="6"/>
-        <v>33.966462264962807</v>
+        <f>O24/O$44*100</f>
+        <v>0.16156872460341609</v>
       </c>
       <c r="U24" s="98"/>
     </row>
-    <row r="25" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
         <v>226</v>
       </c>
@@ -10617,46 +10659,43 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="K25" t="s">
+      <c r="J25" s="136">
+        <v>11</v>
+      </c>
+      <c r="L25" t="s">
         <v>226</v>
       </c>
-      <c r="L25" s="97">
-        <f>(D25)*($O25/100)</f>
+      <c r="M25" s="97">
+        <f>D25*($J25/100)+D37*($J37/100)</f>
         <v>6.6440000000000001</v>
       </c>
-      <c r="M25" s="99">
-        <f>(F25)*($O25/100)</f>
-        <v>0</v>
-      </c>
-      <c r="N25" s="134">
-        <f>(H25)*($O25/100)</f>
-        <v>0</v>
-      </c>
-      <c r="O25" s="140">
-        <v>11</v>
-      </c>
-      <c r="Q25" s="136">
-        <f t="shared" si="3"/>
+      <c r="N25" s="99">
+        <f>F25*($J25/100)+F37*($J37/100)</f>
+        <v>0</v>
+      </c>
+      <c r="O25" s="130">
+        <f>H25*($J25/100)+H37*($J37/100)</f>
+        <v>10.4574</v>
+      </c>
+      <c r="Q25" s="132">
+        <f>M25/M$44*100</f>
         <v>0.59612721878837949</v>
       </c>
       <c r="R25" s="98">
-        <f t="shared" si="4"/>
+        <f>N25/N$44*100</f>
         <v>0</v>
       </c>
       <c r="S25" s="98">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <f>O25/O$44*100</f>
+        <v>4.6933021685215648</v>
       </c>
       <c r="T25" s="102">
-        <f t="shared" si="6"/>
-        <v>0</v>
+        <f>O25/O$44*100</f>
+        <v>4.6933021685215648</v>
       </c>
       <c r="U25" s="98"/>
-      <c r="V25" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="26" spans="1:26" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
         <v>211</v>
       </c>
@@ -10684,46 +10723,43 @@
         <f t="shared" si="2"/>
         <v>5.8582308142940832E-4</v>
       </c>
-      <c r="K26" t="s">
+      <c r="J26" s="136">
+        <v>76</v>
+      </c>
+      <c r="L26" t="s">
         <v>211</v>
       </c>
-      <c r="L26" s="97">
-        <f>(D26)*($O26/100)</f>
+      <c r="M26" s="97">
+        <f>D26*($J26/100)</f>
         <v>3.9520000000000004</v>
       </c>
-      <c r="M26" s="99">
-        <f>(F26)*($O26/100)</f>
-        <v>0</v>
-      </c>
-      <c r="N26" s="134">
-        <f>(H26)*($O26/100)</f>
+      <c r="N26" s="99">
+        <f>F26*($J26/100)</f>
+        <v>0</v>
+      </c>
+      <c r="O26" s="130">
+        <f>H26*($J26/100)</f>
         <v>0.22799999999999998</v>
       </c>
-      <c r="O26" s="140">
-        <v>76</v>
-      </c>
-      <c r="Q26" s="136">
-        <f t="shared" si="3"/>
+      <c r="Q26" s="132">
+        <f>M26/M$44*100</f>
         <v>0.35458982068809092</v>
       </c>
       <c r="R26" s="98">
-        <f t="shared" si="4"/>
+        <f>N26/N$44*100</f>
         <v>0</v>
       </c>
       <c r="S26" s="98">
-        <f t="shared" si="5"/>
-        <v>7.1350224768854983E-2</v>
+        <f>O26/O$44*100</f>
+        <v>0.10232685891549684</v>
       </c>
       <c r="T26" s="102">
-        <f t="shared" si="6"/>
-        <v>7.1350224768854983E-2</v>
+        <f>O26/O$44*100</f>
+        <v>0.10232685891549684</v>
       </c>
       <c r="U26" s="98"/>
-      <c r="V26" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="27" spans="1:26" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
         <v>212</v>
       </c>
@@ -10751,43 +10787,43 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="K27" t="s">
+      <c r="J27" s="136">
+        <v>89</v>
+      </c>
+      <c r="L27" t="s">
         <v>212</v>
       </c>
-      <c r="L27" s="97">
-        <f>(D27)*($O27/100)</f>
+      <c r="M27" s="97">
+        <f>D27*($J27/100)</f>
         <v>7.7429999999999994</v>
       </c>
-      <c r="M27" s="99">
-        <f>(F27)*($O27/100)</f>
-        <v>0</v>
-      </c>
-      <c r="N27" s="134">
-        <f>(H27)*($O27/100)</f>
-        <v>0</v>
-      </c>
-      <c r="O27" s="140">
-        <v>89</v>
-      </c>
-      <c r="Q27" s="136">
-        <f t="shared" si="3"/>
+      <c r="N27" s="99">
+        <f>F27*($J27/100)</f>
+        <v>0</v>
+      </c>
+      <c r="O27" s="130">
+        <f>H27*($J27/100)</f>
+        <v>0</v>
+      </c>
+      <c r="Q27" s="132">
+        <f>M27/M$44*100</f>
         <v>0.69473405404551813</v>
       </c>
       <c r="R27" s="98">
-        <f t="shared" si="4"/>
+        <f>N27/N$44*100</f>
         <v>0</v>
       </c>
       <c r="S27" s="98">
-        <f t="shared" si="5"/>
+        <f>O27/O$44*100</f>
         <v>0</v>
       </c>
       <c r="T27" s="102">
-        <f t="shared" si="6"/>
+        <f>O27/O$44*100</f>
         <v>0</v>
       </c>
       <c r="U27" s="98"/>
     </row>
-    <row r="28" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
         <v>227</v>
       </c>
@@ -10815,45 +10851,45 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="K28" t="s">
+      <c r="J28" s="136">
+        <v>6.3</v>
+      </c>
+      <c r="L28" t="s">
         <v>227</v>
       </c>
-      <c r="L28" s="97">
-        <f>(D28+D38)*($O28/100)</f>
+      <c r="M28" s="97">
+        <f>D28*($J28/100)+D38*($J38/100)</f>
         <v>11.869200000000001</v>
       </c>
-      <c r="M28" s="99">
-        <f>(F28+F38)*($O28/100)</f>
+      <c r="N28" s="99">
+        <f>F28*($J28/100)+F38*($J38/100)</f>
         <v>0.6048</v>
       </c>
-      <c r="N28" s="134">
-        <f>(H28+H38)*($O28/100)</f>
-        <v>7.8434999999999997</v>
-      </c>
-      <c r="O28" s="140">
-        <v>6.3</v>
-      </c>
-      <c r="Q28" s="136">
-        <f t="shared" si="3"/>
+      <c r="O28" s="130">
+        <f>H28*($J28/100)+H38*($J38/100)</f>
+        <v>9.7110000000000003</v>
+      </c>
+      <c r="Q28" s="132">
+        <f>M28/M$44*100</f>
         <v>1.0649538207770974</v>
       </c>
       <c r="R28" s="98">
-        <f t="shared" si="4"/>
+        <f>N28/N$44*100</f>
         <v>1.7626075400433656</v>
       </c>
       <c r="S28" s="98">
-        <f t="shared" si="5"/>
-        <v>2.4545416139233072</v>
+        <f>O28/O$44*100</f>
+        <v>4.3583163461771495</v>
       </c>
       <c r="T28" s="102">
-        <f t="shared" si="6"/>
-        <v>2.4545416139233072</v>
+        <f>O28/O$44*100</f>
+        <v>4.3583163461771495</v>
       </c>
       <c r="U28" s="98"/>
     </row>
-    <row r="29" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="C29" s="109" t="s">
         <v>193</v>
@@ -10879,46 +10915,43 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="K29" t="s">
-        <v>241</v>
-      </c>
-      <c r="L29" s="97">
-        <f>(D29)*($O29/100)</f>
-        <v>0</v>
-      </c>
-      <c r="M29" s="99">
-        <f>(F29)*($O29/100)</f>
+      <c r="J29" s="136">
+        <v>97</v>
+      </c>
+      <c r="L29" t="s">
+        <v>231</v>
+      </c>
+      <c r="M29" s="97">
+        <f>D29*($J29/100)</f>
+        <v>0</v>
+      </c>
+      <c r="N29" s="99">
+        <f>F29*($J29/100)</f>
         <v>9.7000000000000003E-2</v>
       </c>
-      <c r="N29" s="134">
-        <f>(H29)*($O29/100)</f>
-        <v>0</v>
-      </c>
-      <c r="O29" s="140">
-        <v>97</v>
-      </c>
-      <c r="Q29" s="136">
-        <f t="shared" si="3"/>
+      <c r="O29" s="130">
+        <f>H29*($J29/100)</f>
+        <v>0</v>
+      </c>
+      <c r="Q29" s="132">
+        <f>M29/M$44*100</f>
         <v>0</v>
       </c>
       <c r="R29" s="98">
-        <f t="shared" si="4"/>
+        <f>N29/N$44*100</f>
         <v>0.2826933389289128</v>
       </c>
       <c r="S29" s="98">
-        <f t="shared" si="5"/>
+        <f>O29/O$44*100</f>
         <v>0</v>
       </c>
       <c r="T29" s="102">
-        <f t="shared" si="6"/>
+        <f>O29/O$44*100</f>
         <v>0</v>
       </c>
       <c r="U29" s="98"/>
-      <c r="V29" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="30" spans="1:26" x14ac:dyDescent="0.25">
+    </row>
+    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
         <v>223</v>
       </c>
@@ -10946,43 +10979,43 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="K30" t="s">
+      <c r="J30" s="136">
+        <v>92</v>
+      </c>
+      <c r="L30" t="s">
         <v>223</v>
       </c>
-      <c r="L30" s="97">
-        <f>(D30)*($O30/100)</f>
-        <v>0</v>
-      </c>
-      <c r="M30" s="99">
-        <f>(F30)*($O30/100)</f>
+      <c r="M30" s="97">
+        <f>D30*($J30/100)</f>
+        <v>0</v>
+      </c>
+      <c r="N30" s="99">
+        <f>F30*($J30/100)</f>
         <v>0.46</v>
       </c>
-      <c r="N30" s="134">
-        <f>(H30)*($O30/100)</f>
-        <v>0</v>
-      </c>
-      <c r="O30" s="140">
-        <v>92</v>
-      </c>
-      <c r="Q30" s="136">
-        <f t="shared" si="3"/>
+      <c r="O30" s="130">
+        <f>H30*($J30/100)</f>
+        <v>0</v>
+      </c>
+      <c r="Q30" s="132">
+        <f>M30/M$44*100</f>
         <v>0</v>
       </c>
       <c r="R30" s="98">
-        <f t="shared" si="4"/>
+        <f>N30/N$44*100</f>
         <v>1.3406075866731948</v>
       </c>
       <c r="S30" s="98">
-        <f t="shared" si="5"/>
+        <f>O30/O$44*100</f>
         <v>0</v>
       </c>
       <c r="T30" s="102">
-        <f t="shared" si="6"/>
+        <f>O30/O$44*100</f>
         <v>0</v>
       </c>
       <c r="U30" s="98"/>
     </row>
-    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
         <v>224</v>
       </c>
@@ -11010,48 +11043,45 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="K31" t="s">
+      <c r="J31" s="136">
+        <v>92</v>
+      </c>
+      <c r="L31" t="s">
         <v>224</v>
       </c>
-      <c r="L31" s="97">
-        <f>(D31)*($O31/100)</f>
+      <c r="M31" s="97">
+        <f>D31*($J31/100)</f>
         <v>2.0240000000000005</v>
       </c>
-      <c r="M31" s="99">
-        <f>(F31)*($O31/100)</f>
+      <c r="N31" s="99">
+        <f>F31*($J31/100)</f>
         <v>1.1040000000000001</v>
       </c>
-      <c r="N31" s="134">
-        <f>(H31)*($O31/100)</f>
-        <v>0</v>
-      </c>
-      <c r="O31" s="140">
-        <v>92</v>
-      </c>
-      <c r="Q31" s="136">
-        <f t="shared" si="3"/>
+      <c r="O31" s="130">
+        <f>H31*($J31/100)</f>
+        <v>0</v>
+      </c>
+      <c r="Q31" s="132">
+        <f>M31/M$44*100</f>
         <v>0.18160166929977128</v>
       </c>
       <c r="R31" s="98">
-        <f t="shared" si="4"/>
+        <f>N31/N$44*100</f>
         <v>3.2174582080156675</v>
       </c>
       <c r="S31" s="98">
-        <f t="shared" si="5"/>
+        <f>O31/O$44*100</f>
         <v>0</v>
       </c>
       <c r="T31" s="102">
-        <f t="shared" si="6"/>
+        <f>O31/O$44*100</f>
         <v>0</v>
       </c>
       <c r="U31" s="98"/>
-      <c r="V31" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="32" spans="1:26" x14ac:dyDescent="0.25">
+    </row>
+    <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B32" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
       <c r="C32" s="109" t="s">
         <v>197</v>
@@ -11077,144 +11107,136 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="K32" t="s">
-        <v>246</v>
-      </c>
-      <c r="L32" s="97">
-        <f>(D32)*($O32/100)</f>
+      <c r="J32" s="136">
+        <v>100</v>
+      </c>
+      <c r="L32" t="s">
+        <v>236</v>
+      </c>
+      <c r="M32" s="97">
+        <f>D32*($J32/100)</f>
         <v>2.2999999999999998</v>
       </c>
-      <c r="M32" s="99">
-        <f>(F32)*($O32/100)</f>
+      <c r="N32" s="99">
+        <f>F32*($J32/100)</f>
         <v>0.5</v>
       </c>
-      <c r="N32" s="134">
-        <f>(H32)*($O32/100)</f>
-        <v>0</v>
-      </c>
-      <c r="O32" s="140">
-        <v>100</v>
-      </c>
-      <c r="Q32" s="136">
-        <f t="shared" si="3"/>
+      <c r="O32" s="130">
+        <f>H32*($J32/100)</f>
+        <v>0</v>
+      </c>
+      <c r="Q32" s="132">
+        <f>M32/M$44*100</f>
         <v>0.20636553329519458</v>
       </c>
       <c r="R32" s="98">
-        <f t="shared" si="4"/>
+        <f>N32/N$44*100</f>
         <v>1.4571821594273857</v>
       </c>
       <c r="S32" s="98">
-        <f t="shared" si="5"/>
+        <f>O32/O$44*100</f>
         <v>0</v>
       </c>
       <c r="T32" s="102">
-        <f t="shared" si="6"/>
+        <f>O32/O$44*100</f>
         <v>0</v>
       </c>
       <c r="U32" s="98"/>
-      <c r="V32" t="s">
-        <v>238</v>
-      </c>
-      <c r="Z32" t="s">
-        <v>239</v>
-      </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B33" s="87" t="s">
-        <v>253</v>
-      </c>
-      <c r="C33" s="101" t="s">
+        <v>243</v>
+      </c>
+      <c r="C33" s="156" t="s">
         <v>172</v>
       </c>
-      <c r="D33" s="78">
+      <c r="D33" s="157">
         <v>62.6</v>
       </c>
-      <c r="E33" s="110">
+      <c r="E33" s="158">
         <f t="shared" si="0"/>
         <v>3.8430842900116641E-2</v>
       </c>
-      <c r="F33" s="78">
+      <c r="F33" s="157">
         <v>1.8</v>
       </c>
-      <c r="G33" s="110">
+      <c r="G33" s="158">
         <f t="shared" si="1"/>
         <v>3.272727272727273E-2</v>
       </c>
-      <c r="H33" s="78">
+      <c r="H33" s="157">
         <v>11</v>
       </c>
-      <c r="I33" s="111">
+      <c r="I33" s="159">
         <f t="shared" si="2"/>
         <v>2.1480179652411637E-2</v>
       </c>
-      <c r="K33" t="s">
+      <c r="J33" s="136"/>
+      <c r="L33" t="s">
         <v>229</v>
       </c>
-      <c r="L33" s="101">
-        <f>D41</f>
-        <v>0</v>
-      </c>
-      <c r="M33" s="78">
-        <f>F41</f>
-        <v>0</v>
-      </c>
-      <c r="N33" s="100">
-        <f>H41</f>
-        <v>8.8000000000000007</v>
-      </c>
-      <c r="O33" s="140">
-        <v>91</v>
-      </c>
-      <c r="Q33" s="136">
-        <f t="shared" si="3"/>
+      <c r="M33" s="101">
+        <f>D41*($J41/100)</f>
+        <v>0</v>
+      </c>
+      <c r="N33" s="78">
+        <f>F41*($J41/100)</f>
+        <v>0</v>
+      </c>
+      <c r="O33" s="100">
+        <f>H41*($J41/100)</f>
+        <v>7.9200000000000008</v>
+      </c>
+      <c r="Q33" s="132">
+        <f>M33/M$44*100</f>
         <v>0</v>
       </c>
       <c r="R33" s="98">
-        <f t="shared" si="4"/>
+        <f>N33/N$44*100</f>
         <v>0</v>
       </c>
       <c r="S33" s="98">
-        <f t="shared" si="5"/>
-        <v>2.7538683244119473</v>
+        <f>O33/O$44*100</f>
+        <v>3.554511941275154</v>
       </c>
       <c r="T33" s="102">
-        <f t="shared" si="6"/>
-        <v>2.7538683244119473</v>
+        <f>O33/O$44*100</f>
+        <v>3.554511941275154</v>
       </c>
       <c r="U33" s="98"/>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B34" s="87" t="s">
-        <v>253</v>
-      </c>
-      <c r="C34" s="101" t="s">
+        <v>243</v>
+      </c>
+      <c r="C34" s="156" t="s">
         <v>186</v>
       </c>
-      <c r="D34" s="78">
+      <c r="D34" s="157">
         <v>5.8</v>
       </c>
-      <c r="E34" s="110">
+      <c r="E34" s="158">
         <f t="shared" si="0"/>
         <v>3.5606851249309346E-3</v>
       </c>
-      <c r="F34" s="78">
+      <c r="F34" s="157">
         <v>0.2</v>
       </c>
-      <c r="G34" s="110">
+      <c r="G34" s="158">
         <f t="shared" si="1"/>
         <v>3.6363636363636364E-3</v>
       </c>
-      <c r="H34" s="78">
+      <c r="H34" s="157">
         <v>1.4</v>
       </c>
-      <c r="I34" s="111">
+      <c r="I34" s="159">
         <f t="shared" si="2"/>
         <v>2.7338410466705718E-3</v>
       </c>
-      <c r="L34" s="101"/>
-      <c r="M34" s="78"/>
-      <c r="N34" s="100"/>
-      <c r="O34" s="140"/>
+      <c r="J34" s="136"/>
+      <c r="M34" s="101"/>
+      <c r="N34" s="78"/>
+      <c r="O34" s="100"/>
       <c r="Q34" s="101"/>
       <c r="R34" s="78"/>
       <c r="S34" s="78"/>
@@ -11223,36 +11245,36 @@
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B35" s="87" t="s">
-        <v>253</v>
-      </c>
-      <c r="C35" s="101" t="s">
+        <v>243</v>
+      </c>
+      <c r="C35" s="156" t="s">
         <v>201</v>
       </c>
-      <c r="D35" s="78">
+      <c r="D35" s="157">
         <v>43.3</v>
       </c>
-      <c r="E35" s="110">
+      <c r="E35" s="158">
         <f t="shared" si="0"/>
         <v>2.6582356191294735E-2</v>
       </c>
-      <c r="F35" s="78">
+      <c r="F35" s="157">
         <v>4.5</v>
       </c>
-      <c r="G35" s="110">
+      <c r="G35" s="158">
         <f t="shared" si="1"/>
         <v>8.1818181818181818E-2</v>
       </c>
-      <c r="H35" s="78">
-        <v>0</v>
-      </c>
-      <c r="I35" s="111">
+      <c r="H35" s="157">
+        <v>0</v>
+      </c>
+      <c r="I35" s="159">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L35" s="101"/>
-      <c r="M35" s="78"/>
-      <c r="N35" s="100"/>
-      <c r="O35" s="140"/>
+      <c r="J35" s="136"/>
+      <c r="M35" s="101"/>
+      <c r="N35" s="78"/>
+      <c r="O35" s="100"/>
       <c r="Q35" s="101"/>
       <c r="R35" s="78"/>
       <c r="S35" s="78"/>
@@ -11287,10 +11309,12 @@
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="L36" s="101"/>
-      <c r="M36" s="78"/>
-      <c r="N36" s="100"/>
-      <c r="O36" s="140"/>
+      <c r="J36" s="136">
+        <v>86</v>
+      </c>
+      <c r="M36" s="101"/>
+      <c r="N36" s="78"/>
+      <c r="O36" s="100"/>
       <c r="Q36" s="101"/>
       <c r="R36" s="78"/>
       <c r="S36" s="78"/>
@@ -11302,34 +11326,36 @@
       <c r="B37" t="s">
         <v>226</v>
       </c>
-      <c r="C37" s="118" t="s">
+      <c r="C37" s="117" t="s">
         <v>202</v>
       </c>
-      <c r="D37" s="119">
-        <v>0</v>
-      </c>
-      <c r="E37" s="120">
+      <c r="D37" s="118">
+        <v>0</v>
+      </c>
+      <c r="E37" s="119">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F37" s="119">
-        <v>0</v>
-      </c>
-      <c r="G37" s="120">
+      <c r="F37" s="118">
+        <v>0</v>
+      </c>
+      <c r="G37" s="119">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="H37" s="119">
+      <c r="H37" s="118">
         <v>120.2</v>
       </c>
-      <c r="I37" s="121">
+      <c r="I37" s="120">
         <f t="shared" si="2"/>
         <v>0.23471978129271626</v>
       </c>
-      <c r="L37" s="101"/>
-      <c r="M37" s="78"/>
-      <c r="N37" s="100"/>
-      <c r="O37" s="140"/>
+      <c r="J37" s="136">
+        <v>8.6999999999999993</v>
+      </c>
+      <c r="M37" s="101"/>
+      <c r="N37" s="78"/>
+      <c r="O37" s="100"/>
       <c r="Q37" s="101"/>
       <c r="R37" s="78"/>
       <c r="S37" s="78"/>
@@ -11364,10 +11390,12 @@
         <f t="shared" si="2"/>
         <v>0.24311657879320445</v>
       </c>
-      <c r="L38" s="101"/>
-      <c r="M38" s="78"/>
-      <c r="N38" s="100"/>
-      <c r="O38" s="140"/>
+      <c r="J38" s="136">
+        <v>7.8</v>
+      </c>
+      <c r="M38" s="101"/>
+      <c r="N38" s="78"/>
+      <c r="O38" s="100"/>
       <c r="Q38" s="101"/>
       <c r="R38" s="78"/>
       <c r="S38" s="78"/>
@@ -11402,10 +11430,12 @@
         <f t="shared" si="2"/>
         <v>3.4954110525288025E-2</v>
       </c>
-      <c r="L39" s="101"/>
-      <c r="M39" s="78"/>
-      <c r="N39" s="100"/>
-      <c r="O39" s="140"/>
+      <c r="J39" s="136">
+        <v>87</v>
+      </c>
+      <c r="M39" s="101"/>
+      <c r="N39" s="78"/>
+      <c r="O39" s="100"/>
       <c r="Q39" s="101"/>
       <c r="R39" s="78"/>
       <c r="S39" s="78"/>
@@ -11414,36 +11444,38 @@
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B40" s="87" t="s">
-        <v>253</v>
-      </c>
-      <c r="C40" s="112" t="s">
+        <v>243</v>
+      </c>
+      <c r="C40" s="160" t="s">
         <v>205</v>
       </c>
-      <c r="D40" s="78">
-        <v>0</v>
-      </c>
-      <c r="E40" s="110">
+      <c r="D40" s="157">
+        <v>0</v>
+      </c>
+      <c r="E40" s="158">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F40" s="78">
-        <v>0</v>
-      </c>
-      <c r="G40" s="110">
+      <c r="F40" s="157">
+        <v>0</v>
+      </c>
+      <c r="G40" s="158">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="H40" s="78">
+      <c r="H40" s="157">
         <v>15.7</v>
       </c>
-      <c r="I40" s="111">
+      <c r="I40" s="159">
         <f t="shared" si="2"/>
         <v>3.0658074594805698E-2</v>
       </c>
-      <c r="L40" s="101"/>
-      <c r="M40" s="78"/>
-      <c r="N40" s="100"/>
-      <c r="O40" s="140"/>
+      <c r="J40" s="136">
+        <v>91</v>
+      </c>
+      <c r="M40" s="101"/>
+      <c r="N40" s="78"/>
+      <c r="O40" s="100"/>
       <c r="Q40" s="101"/>
       <c r="R40" s="78"/>
       <c r="S40" s="78"/>
@@ -11478,10 +11510,12 @@
         <f t="shared" si="2"/>
         <v>1.718414372192931E-2</v>
       </c>
-      <c r="L41" s="101"/>
-      <c r="M41" s="78"/>
-      <c r="N41" s="100"/>
-      <c r="O41" s="140"/>
+      <c r="J41" s="136">
+        <v>90</v>
+      </c>
+      <c r="M41" s="101"/>
+      <c r="N41" s="78"/>
+      <c r="O41" s="100"/>
       <c r="Q41" s="101"/>
       <c r="R41" s="78"/>
       <c r="S41" s="78"/>
@@ -11490,36 +11524,36 @@
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="B42" s="87" t="s">
-        <v>253</v>
-      </c>
-      <c r="C42" s="122" t="s">
+        <v>243</v>
+      </c>
+      <c r="C42" s="161" t="s">
         <v>207</v>
       </c>
-      <c r="D42" s="76">
-        <v>0</v>
-      </c>
-      <c r="E42" s="123">
+      <c r="D42" s="162">
+        <v>0</v>
+      </c>
+      <c r="E42" s="163">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="F42" s="76">
-        <v>0</v>
-      </c>
-      <c r="G42" s="123">
+      <c r="F42" s="162">
+        <v>0</v>
+      </c>
+      <c r="G42" s="163">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="H42" s="76">
+      <c r="H42" s="162">
         <v>4.7</v>
       </c>
-      <c r="I42" s="124">
+      <c r="I42" s="164">
         <f t="shared" si="2"/>
         <v>9.1778949423940628E-3</v>
       </c>
-      <c r="L42" s="101"/>
-      <c r="M42" s="78"/>
-      <c r="N42" s="100"/>
-      <c r="O42" s="140"/>
+      <c r="J42" s="136"/>
+      <c r="M42" s="101"/>
+      <c r="N42" s="78"/>
+      <c r="O42" s="100"/>
       <c r="Q42" s="101"/>
       <c r="R42" s="78"/>
       <c r="S42" s="78"/>
@@ -11527,7 +11561,7 @@
       <c r="U42" s="78"/>
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="C43" s="125" t="s">
+      <c r="C43" s="121" t="s">
         <v>198</v>
       </c>
       <c r="D43" s="77">
@@ -11541,11 +11575,11 @@
       <c r="H43" s="77">
         <v>330.2</v>
       </c>
-      <c r="I43" s="126"/>
-      <c r="L43" s="101"/>
-      <c r="M43" s="78"/>
-      <c r="N43" s="100"/>
-      <c r="O43" s="140"/>
+      <c r="I43" s="122"/>
+      <c r="J43" s="136"/>
+      <c r="M43" s="101"/>
+      <c r="N43" s="78"/>
+      <c r="O43" s="100"/>
       <c r="Q43" s="101"/>
       <c r="R43" s="78"/>
       <c r="S43" s="78"/>
@@ -11556,114 +11590,139 @@
       <c r="C44" s="107" t="s">
         <v>208</v>
       </c>
-      <c r="D44" s="113">
+      <c r="D44" s="112">
         <v>4375.1000000000004</v>
       </c>
-      <c r="E44" s="113"/>
-      <c r="F44" s="113">
+      <c r="E44" s="112"/>
+      <c r="F44" s="112">
         <v>134.9</v>
       </c>
-      <c r="G44" s="113"/>
-      <c r="H44" s="113">
+      <c r="G44" s="112"/>
+      <c r="H44" s="112">
         <v>842.3</v>
       </c>
-      <c r="I44" s="114"/>
-      <c r="K44" s="4" t="s">
-        <v>247</v>
-      </c>
-      <c r="L44" s="127">
-        <f>SUM(L8:L43)</f>
+      <c r="I44" s="113"/>
+      <c r="J44" s="136"/>
+      <c r="L44" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="M44" s="123">
+        <f>SUM(M8:M43)</f>
         <v>1114.5272</v>
       </c>
-      <c r="M44" s="137">
-        <f>SUM(M8:M43)</f>
+      <c r="N44" s="133">
+        <f>SUM(N8:N43)</f>
         <v>34.312800000000003</v>
       </c>
-      <c r="N44" s="128">
-        <f>SUM(N8:N43)</f>
-        <v>319.55050000000006</v>
-      </c>
-      <c r="O44" s="140"/>
-      <c r="Q44" s="127">
+      <c r="O44" s="124">
+        <f>SUM(O8:O43)</f>
+        <v>222.81540000000004</v>
+      </c>
+      <c r="Q44" s="123">
         <f>SUM(Q8:Q43)</f>
         <v>100</v>
       </c>
-      <c r="R44" s="137">
-        <f t="shared" ref="R44:T44" si="10">SUM(R8:R43)</f>
+      <c r="R44" s="133">
+        <f t="shared" ref="R44:T44" si="3">SUM(R8:R43)</f>
         <v>100</v>
       </c>
-      <c r="S44" s="137">
-        <f t="shared" si="10"/>
-        <v>99.999999999999986</v>
-      </c>
-      <c r="T44" s="128">
-        <f t="shared" si="10"/>
-        <v>99.999999999999986</v>
-      </c>
-      <c r="U44" s="133"/>
+      <c r="S44" s="133">
+        <f t="shared" si="3"/>
+        <v>100</v>
+      </c>
+      <c r="T44" s="124">
+        <f t="shared" si="3"/>
+        <v>100</v>
+      </c>
+      <c r="U44" s="129"/>
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="C45" s="115" t="s">
+      <c r="C45" s="114" t="s">
         <v>228</v>
       </c>
-      <c r="D45" s="116">
+      <c r="D45" s="115">
         <f>SUM(D8:D42)</f>
         <v>1628.9</v>
       </c>
-      <c r="E45" s="116"/>
-      <c r="F45" s="116">
+      <c r="E45" s="115"/>
+      <c r="F45" s="115">
         <f>SUM(F8:F42)</f>
         <v>55</v>
       </c>
-      <c r="G45" s="116"/>
-      <c r="H45" s="116">
+      <c r="G45" s="115"/>
+      <c r="H45" s="115">
         <f>SUM(H8:H42)</f>
         <v>512.1</v>
       </c>
-      <c r="I45" s="117"/>
+      <c r="I45" s="116"/>
+      <c r="J45" s="136"/>
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="K46" s="103"/>
-      <c r="L46" s="87"/>
+      <c r="L46" s="103"/>
       <c r="M46" s="87"/>
       <c r="N46" s="87"/>
+      <c r="O46" s="87"/>
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="C47" s="141" t="s">
-        <v>251</v>
-      </c>
-      <c r="K47" s="103"/>
-      <c r="L47" s="87"/>
+      <c r="C47" s="137" t="s">
+        <v>241</v>
+      </c>
+      <c r="L47" s="103"/>
       <c r="M47" s="87"/>
       <c r="N47" s="87"/>
+      <c r="O47" s="87"/>
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="C48" s="141" t="s">
-        <v>252</v>
-      </c>
-      <c r="K48" s="103"/>
-      <c r="L48" s="87"/>
+      <c r="C48" s="137" t="s">
+        <v>242</v>
+      </c>
+      <c r="L48" s="103"/>
       <c r="M48" s="87"/>
       <c r="N48" s="87"/>
-    </row>
-    <row r="49" spans="11:14" x14ac:dyDescent="0.25">
-      <c r="K49" s="87"/>
+      <c r="O48" s="87"/>
+    </row>
+    <row r="49" spans="3:15" x14ac:dyDescent="0.25">
       <c r="L49" s="87"/>
       <c r="M49" s="87"/>
       <c r="N49" s="87"/>
-    </row>
-    <row r="50" spans="11:14" x14ac:dyDescent="0.25">
-      <c r="K50" s="103"/>
-      <c r="L50" s="87"/>
+      <c r="O49" s="87"/>
+    </row>
+    <row r="50" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="L50" s="103"/>
       <c r="M50" s="87"/>
       <c r="N50" s="87"/>
+      <c r="O50" s="87"/>
+    </row>
+    <row r="51" spans="3:15" x14ac:dyDescent="0.25">
+      <c r="C51" s="150" t="s">
+        <v>245</v>
+      </c>
+      <c r="D51" s="118"/>
+      <c r="E51" s="118"/>
+      <c r="F51" s="118"/>
+      <c r="G51" s="118"/>
+      <c r="H51" s="118"/>
+      <c r="I51" s="151"/>
+      <c r="J51" s="78"/>
+    </row>
+    <row r="52" spans="3:15" ht="91.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C52" s="152" t="s">
+        <v>244</v>
+      </c>
+      <c r="D52" s="153"/>
+      <c r="E52" s="153"/>
+      <c r="F52" s="153"/>
+      <c r="G52" s="153"/>
+      <c r="H52" s="153"/>
+      <c r="I52" s="154"/>
+      <c r="J52" s="155"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="V7" r:id="rId1"/>
-  </hyperlinks>
+  <mergeCells count="1">
+    <mergeCell ref="C52:I52"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -13915,19 +13974,19 @@
     </row>
     <row r="23" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B23" s="40"/>
-      <c r="C23" s="148" t="s">
+      <c r="C23" s="144" t="s">
         <v>97</v>
       </c>
-      <c r="D23" s="150" t="s">
+      <c r="D23" s="146" t="s">
         <v>86</v>
       </c>
-      <c r="E23" s="143" t="s">
+      <c r="E23" s="139" t="s">
         <v>87</v>
       </c>
-      <c r="F23" s="145" t="s">
+      <c r="F23" s="141" t="s">
         <v>92</v>
       </c>
-      <c r="G23" s="147"/>
+      <c r="G23" s="143"/>
       <c r="H23" s="31"/>
       <c r="O23">
         <v>11</v>
@@ -13949,11 +14008,11 @@
     </row>
     <row r="24" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B24" s="41"/>
-      <c r="C24" s="149"/>
-      <c r="D24" s="151"/>
-      <c r="E24" s="144"/>
-      <c r="F24" s="146"/>
-      <c r="G24" s="147"/>
+      <c r="C24" s="145"/>
+      <c r="D24" s="147"/>
+      <c r="E24" s="140"/>
+      <c r="F24" s="142"/>
+      <c r="G24" s="143"/>
       <c r="H24" s="18"/>
       <c r="O24">
         <v>13</v>
@@ -13974,13 +14033,13 @@
       </c>
     </row>
     <row r="25" spans="2:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="153" t="s">
+      <c r="B25" s="149" t="s">
         <v>9</v>
       </c>
-      <c r="C25" s="153"/>
-      <c r="D25" s="153"/>
-      <c r="E25" s="153"/>
-      <c r="F25" s="153"/>
+      <c r="C25" s="149"/>
+      <c r="D25" s="149"/>
+      <c r="E25" s="149"/>
+      <c r="F25" s="149"/>
       <c r="G25" s="42"/>
       <c r="H25" s="18"/>
       <c r="O25">
@@ -14002,13 +14061,13 @@
       </c>
     </row>
     <row r="26" spans="2:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="142" t="s">
+      <c r="B26" s="138" t="s">
         <v>93</v>
       </c>
-      <c r="C26" s="142"/>
-      <c r="D26" s="142"/>
-      <c r="E26" s="142"/>
-      <c r="F26" s="142"/>
+      <c r="C26" s="138"/>
+      <c r="D26" s="138"/>
+      <c r="E26" s="138"/>
+      <c r="F26" s="138"/>
       <c r="G26" s="42"/>
       <c r="H26" s="18"/>
       <c r="O26">
@@ -14200,25 +14259,25 @@
       <c r="R33" s="3"/>
     </row>
     <row r="34" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="152" t="s">
+      <c r="B34" s="148" t="s">
         <v>8</v>
       </c>
-      <c r="C34" s="152"/>
-      <c r="D34" s="152"/>
-      <c r="E34" s="152"/>
-      <c r="F34" s="152"/>
+      <c r="C34" s="148"/>
+      <c r="D34" s="148"/>
+      <c r="E34" s="148"/>
+      <c r="F34" s="148"/>
       <c r="G34" s="42"/>
       <c r="H34" s="18"/>
       <c r="R34" s="13"/>
     </row>
     <row r="35" spans="2:18" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="142" t="s">
+      <c r="B35" s="138" t="s">
         <v>94</v>
       </c>
-      <c r="C35" s="142"/>
-      <c r="D35" s="142"/>
-      <c r="E35" s="142"/>
-      <c r="F35" s="142"/>
+      <c r="C35" s="138"/>
+      <c r="D35" s="138"/>
+      <c r="E35" s="138"/>
+      <c r="F35" s="138"/>
       <c r="G35" s="42"/>
       <c r="H35" s="18"/>
     </row>

</xml_diff>